<commit_message>
Stage 1 ready for DT integration
Signed-off-by: Aytug <aytug.yavuzer@eonerc.rwth-aachen.de>
</commit_message>
<xml_diff>
--- a/inputs/acceptance_cases/stage1_baseline_multi_cluster.xlsx
+++ b/inputs/acceptance_cases/stage1_baseline_multi_cluster.xlsx
@@ -10,6 +10,7 @@
     <sheet name="Planning" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Fleet" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Clusters" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="DayAheadMarketPrices" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -578,7 +579,7 @@
         <v>1</v>
       </c>
       <c r="J2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K2" t="n">
         <v>0</v>
@@ -621,7 +622,7 @@
         <v>1</v>
       </c>
       <c r="J3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K3" t="n">
         <v>0</v>
@@ -664,7 +665,7 @@
         <v>1</v>
       </c>
       <c r="J4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K4" t="n">
         <v>0</v>
@@ -707,7 +708,7 @@
         <v>1</v>
       </c>
       <c r="J5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K5" t="n">
         <v>0.2</v>
@@ -750,7 +751,7 @@
         <v>1</v>
       </c>
       <c r="J6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K6" t="n">
         <v>0.2</v>
@@ -793,7 +794,7 @@
         <v>1</v>
       </c>
       <c r="J7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K7" t="n">
         <v>0.2</v>
@@ -879,7 +880,7 @@
         <v>1</v>
       </c>
       <c r="J9" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K9" t="n">
         <v>0</v>
@@ -922,7 +923,7 @@
         <v>1</v>
       </c>
       <c r="J10" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K10" t="n">
         <v>0</v>
@@ -1149,4 +1150,222 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B25"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>timestamp</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>price_eur_per_kwh</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="n">
+        <v>44569.29166666666</v>
+      </c>
+      <c r="B2" t="n">
+        <v>0.28</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="n">
+        <v>44569.30208333334</v>
+      </c>
+      <c r="B3" t="n">
+        <v>0.27</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="n">
+        <v>44569.3125</v>
+      </c>
+      <c r="B4" t="n">
+        <v>0.26</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="n">
+        <v>44569.32291666666</v>
+      </c>
+      <c r="B5" t="n">
+        <v>0.24</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="n">
+        <v>44569.33333333334</v>
+      </c>
+      <c r="B6" t="n">
+        <v>0.22</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="n">
+        <v>44569.34375</v>
+      </c>
+      <c r="B7" t="n">
+        <v>0.2</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="n">
+        <v>44569.35416666666</v>
+      </c>
+      <c r="B8" t="n">
+        <v>0.18</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="n">
+        <v>44569.36458333334</v>
+      </c>
+      <c r="B9" t="n">
+        <v>0.16</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="n">
+        <v>44569.375</v>
+      </c>
+      <c r="B10" t="n">
+        <v>0.15</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="n">
+        <v>44569.38541666666</v>
+      </c>
+      <c r="B11" t="n">
+        <v>0.14</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="n">
+        <v>44569.39583333334</v>
+      </c>
+      <c r="B12" t="n">
+        <v>0.13</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="n">
+        <v>44569.40625</v>
+      </c>
+      <c r="B13" t="n">
+        <v>0.12</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="n">
+        <v>44569.41666666666</v>
+      </c>
+      <c r="B14" t="n">
+        <v>0.11</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="n">
+        <v>44569.42708333334</v>
+      </c>
+      <c r="B15" t="n">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="n">
+        <v>44569.4375</v>
+      </c>
+      <c r="B16" t="n">
+        <v>0.11</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="n">
+        <v>44569.44791666666</v>
+      </c>
+      <c r="B17" t="n">
+        <v>0.12</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="n">
+        <v>44569.45833333334</v>
+      </c>
+      <c r="B18" t="n">
+        <v>0.14</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="n">
+        <v>44569.46875</v>
+      </c>
+      <c r="B19" t="n">
+        <v>0.16</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="n">
+        <v>44569.47916666666</v>
+      </c>
+      <c r="B20" t="n">
+        <v>0.18</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="n">
+        <v>44569.48958333334</v>
+      </c>
+      <c r="B21" t="n">
+        <v>0.2</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="n">
+        <v>44569.5</v>
+      </c>
+      <c r="B22" t="n">
+        <v>0.22</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="n">
+        <v>44569.51041666666</v>
+      </c>
+      <c r="B23" t="n">
+        <v>0.24</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="n">
+        <v>44569.52083333334</v>
+      </c>
+      <c r="B24" t="n">
+        <v>0.26</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="n">
+        <v>44569.53125</v>
+      </c>
+      <c r="B25" t="n">
+        <v>0.28</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>